<commit_message>
Set device maintenance status log ID on each device in demo seeds
</commit_message>
<xml_diff>
--- a/api/templates/device_activity_percent/en.xlsx
+++ b/api/templates/device_activity_percent/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bryan\projects\SystemOne\aspect\api\templates\device_activity_percent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213F8465-D975-476E-A165-C69F214BDA6E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4691E6E9-3826-4A41-AFF4-7FF80EE62C1A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="27634" windowHeight="15034" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activity (Percent)" sheetId="1" r:id="rId1"/>
@@ -584,56 +584,56 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="31.875" customWidth="1"/>
-    <col min="2" max="2" width="26.375" customWidth="1"/>
-    <col min="3" max="3" width="18.125" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.35546875" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" customWidth="1"/>
     <col min="4" max="4" width="29.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
@@ -650,7 +650,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>